<commit_message>
Updates following USNA Meeting - I
</commit_message>
<xml_diff>
--- a/EPN_facilities.xlsx
+++ b/EPN_facilities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sushreyomisra07/Documents/GitHub/FloodRiskBTP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2AE81A4-4A6F-C84C-AC01-24ECFB3C9BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{142A287E-C5C9-FA48-83DD-99A5BB808882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="19200" windowHeight="11380" activeTab="2" xr2:uid="{7713A25D-7047-4BE5-B59D-81615470B2F5}"/>
+    <workbookView xWindow="1860" yWindow="500" windowWidth="26580" windowHeight="17960" activeTab="2" xr2:uid="{7713A25D-7047-4BE5-B59D-81615470B2F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Power_Plants" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Updates after USNA meeting - II
</commit_message>
<xml_diff>
--- a/EPN_facilities.xlsx
+++ b/EPN_facilities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sushreyomisra07/Documents/GitHub/FloodRiskBTP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{142A287E-C5C9-FA48-83DD-99A5BB808882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE3B1A0-45BE-2C4E-801D-4834F2630D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="500" windowWidth="26580" windowHeight="17960" activeTab="2" xr2:uid="{7713A25D-7047-4BE5-B59D-81615470B2F5}"/>
+    <workbookView xWindow="1860" yWindow="760" windowWidth="26580" windowHeight="17900" activeTab="1" xr2:uid="{7713A25D-7047-4BE5-B59D-81615470B2F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Power_Plants" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="42">
   <si>
     <t>Herbert A Wagner Generating Station</t>
   </si>
@@ -159,7 +159,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,6 +172,13 @@
       <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -194,9 +201,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,10 +519,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6FED44D-86D4-46E9-9B58-F887B4AA0D54}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -528,10 +536,13 @@
         <v>6</v>
       </c>
       <c r="E1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -544,11 +555,14 @@
       <c r="D2">
         <v>-76.441607000000005</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -561,7 +575,10 @@
       <c r="D3">
         <v>-76.525818999999998</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -572,13 +589,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{484B7608-B400-49F9-98B0-0A52DF03BAEC}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -594,11 +612,14 @@
       <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>3</v>
       </c>
@@ -614,11 +635,14 @@
       <c r="E2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>4</v>
       </c>
@@ -635,10 +659,13 @@
         <v>15</v>
       </c>
       <c r="F3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>5</v>
       </c>
@@ -655,10 +682,13 @@
         <v>15</v>
       </c>
       <c r="F4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>6</v>
       </c>
@@ -675,10 +705,13 @@
         <v>15</v>
       </c>
       <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>7</v>
       </c>
@@ -695,10 +728,13 @@
         <v>15</v>
       </c>
       <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>8</v>
       </c>
@@ -715,6 +751,9 @@
         <v>15</v>
       </c>
       <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
         <v>1</v>
       </c>
     </row>

</xml_diff>